<commit_message>
Running Andrew's changes and adding the distribution data
</commit_message>
<xml_diff>
--- a/data/nameFixes.xlsx
+++ b/data/nameFixes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahipp\Documents\github\herbphenology2026\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/miriamhafkin/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431DFC26-212E-41C2-8E7D-243CB0EE0A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30222154-92E1-954B-B0E9-2C5331D7FFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{E9156B2C-06D0-4B0A-BE5A-4E91FB64ACDF}"/>
+    <workbookView xWindow="5460" yWindow="760" windowWidth="14240" windowHeight="11460" xr2:uid="{E9156B2C-06D0-4B0A-BE5A-4E91FB64ACDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>original</t>
   </si>
@@ -88,6 +88,12 @@
   </si>
   <si>
     <t>Acer platanoides subsp. turkestanicum (Pax) P.C.de Jong</t>
+  </si>
+  <si>
+    <t>Acer barbatum Michx.</t>
+  </si>
+  <si>
+    <t>Acer saccharum subsp. Floridanum (Chapm.)</t>
   </si>
 </sst>
 </file>
@@ -143,9 +149,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -183,7 +189,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -289,7 +295,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -431,7 +437,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -439,14 +445,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB294A23-2077-47B9-B6A8-0013F1CE80D7}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -457,7 +463,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -468,46 +474,54 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A4" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A5" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A6" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>13</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="A7" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>15</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>